<commit_message>
Add CO2 abatement cost to Pareto-front grid
Marginal abatement cost ($/tCO2) vs grey base (x0, CCS0), E=31.66 MJ/L, same
formula as tea_scale_up_abatement.py. New abatement column in xlsx; report §5
front table. Grey+CCS 25-50% cheapest (~165 $/t); green-NH3 tail 485-888 $/t.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CaRxY6dB1J1eEsJrcJqdte
</commit_message>
<xml_diff>
--- a/Result/pareto_front.xlsx
+++ b/Result/pareto_front.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F31"/>
+  <dimension ref="A1:G31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -459,6 +459,11 @@
           <t>pareto</t>
         </is>
       </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>abatement</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -479,6 +484,7 @@
       <c r="F2" t="b">
         <v>1</v>
       </c>
+      <c r="G2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -499,6 +505,9 @@
       <c r="F3" t="b">
         <v>1</v>
       </c>
+      <c r="G3" t="n">
+        <v>169.4958</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -519,6 +528,9 @@
       <c r="F4" t="b">
         <v>1</v>
       </c>
+      <c r="G4" t="n">
+        <v>164.735</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -539,6 +551,9 @@
       <c r="F5" t="b">
         <v>1</v>
       </c>
+      <c r="G5" t="n">
+        <v>301.3643</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -559,6 +574,9 @@
       <c r="F6" t="b">
         <v>1</v>
       </c>
+      <c r="G6" t="n">
+        <v>393.6594</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -579,6 +597,9 @@
       <c r="F7" t="b">
         <v>0</v>
       </c>
+      <c r="G7" t="n">
+        <v>1528.1643</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -599,6 +620,9 @@
       <c r="F8" t="b">
         <v>0</v>
       </c>
+      <c r="G8" t="n">
+        <v>506.3655</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -619,6 +643,9 @@
       <c r="F9" t="b">
         <v>1</v>
       </c>
+      <c r="G9" t="n">
+        <v>357.6029</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -639,6 +666,9 @@
       <c r="F10" t="b">
         <v>1</v>
       </c>
+      <c r="G10" t="n">
+        <v>427.0394</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -658,6 +688,9 @@
       </c>
       <c r="F11" t="b">
         <v>1</v>
+      </c>
+      <c r="G11" t="n">
+        <v>485.2141</v>
       </c>
     </row>
     <row r="12">
@@ -679,6 +712,9 @@
       <c r="F12" t="b">
         <v>0</v>
       </c>
+      <c r="G12" t="n">
+        <v>1484.4588</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -699,6 +735,9 @@
       <c r="F13" t="b">
         <v>0</v>
       </c>
+      <c r="G13" t="n">
+        <v>763.6181</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -719,6 +758,9 @@
       <c r="F14" t="b">
         <v>0</v>
       </c>
+      <c r="G14" t="n">
+        <v>549.7527</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -739,6 +781,9 @@
       <c r="F15" t="b">
         <v>0</v>
       </c>
+      <c r="G15" t="n">
+        <v>564.0014</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -759,6 +804,9 @@
       <c r="F16" t="b">
         <v>1</v>
       </c>
+      <c r="G16" t="n">
+        <v>589.9656</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -779,6 +827,9 @@
       <c r="F17" t="b">
         <v>0</v>
       </c>
+      <c r="G17" t="n">
+        <v>1470.1692</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -799,6 +850,9 @@
       <c r="F18" t="b">
         <v>0</v>
       </c>
+      <c r="G18" t="n">
+        <v>979.0553</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -819,6 +873,9 @@
       <c r="F19" t="b">
         <v>0</v>
       </c>
+      <c r="G19" t="n">
+        <v>754.4023999999999</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -839,6 +896,9 @@
       <c r="F20" t="b">
         <v>0</v>
       </c>
+      <c r="G20" t="n">
+        <v>726.0234</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -859,6 +919,9 @@
       <c r="F21" t="b">
         <v>1</v>
       </c>
+      <c r="G21" t="n">
+        <v>722.0327</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -879,6 +942,9 @@
       <c r="F22" t="b">
         <v>0</v>
       </c>
+      <c r="G22" t="n">
+        <v>1462.1736</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -899,6 +965,9 @@
       <c r="F23" t="b">
         <v>0</v>
       </c>
+      <c r="G23" t="n">
+        <v>1089.9253</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -919,6 +988,9 @@
       <c r="F24" t="b">
         <v>0</v>
       </c>
+      <c r="G24" t="n">
+        <v>881.8561999999999</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -939,6 +1011,9 @@
       <c r="F25" t="b">
         <v>0</v>
       </c>
+      <c r="G25" t="n">
+        <v>836.7375</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -959,6 +1034,9 @@
       <c r="F26" t="b">
         <v>1</v>
       </c>
+      <c r="G26" t="n">
+        <v>817.8625</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -979,6 +1057,9 @@
       <c r="F27" t="b">
         <v>0</v>
       </c>
+      <c r="G27" t="n">
+        <v>1451.3225</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -999,6 +1080,9 @@
       <c r="F28" t="b">
         <v>0</v>
       </c>
+      <c r="G28" t="n">
+        <v>1153.0033</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -1019,6 +1103,9 @@
       <c r="F29" t="b">
         <v>0</v>
       </c>
+      <c r="G29" t="n">
+        <v>965.3873</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -1039,6 +1126,9 @@
       <c r="F30" t="b">
         <v>0</v>
       </c>
+      <c r="G30" t="n">
+        <v>914.2934</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -1058,6 +1148,9 @@
       </c>
       <c r="F31" t="b">
         <v>1</v>
+      </c>
+      <c r="G31" t="n">
+        <v>888.0896</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Rebase Pareto CO2 abatement cost onto the CORSIA-compliance floor
Reference abatement to the cheapest CORSIA-compliant point (grey H2 +
CCS25, 76.0 g/MJ ~ 0.9x conventional) instead of the grey base. The
floor is the 0 $/tCO2 reference (colored on the contour); only cells
strictly dirtier than the floor are n/a. New compliance-floor contour
Figure/pareto_abatement_contour_compliance.png; old grey-base contour
and report section 5 history kept. _Pareto_Front.md sections 3/5 + log
updated.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012zMKU1n4MNK6d4dYMH2ipe
</commit_message>
<xml_diff>
--- a/Result/pareto_front.xlsx
+++ b/Result/pareto_front.xlsx
@@ -506,7 +506,7 @@
         <v>1</v>
       </c>
       <c r="G3" t="n">
-        <v>169.4958</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4">
@@ -529,7 +529,7 @@
         <v>1</v>
       </c>
       <c r="G4" t="n">
-        <v>164.735</v>
+        <v>159.9786</v>
       </c>
     </row>
     <row r="5">
@@ -552,7 +552,7 @@
         <v>1</v>
       </c>
       <c r="G5" t="n">
-        <v>301.3643</v>
+        <v>371.1885</v>
       </c>
     </row>
     <row r="6">
@@ -575,7 +575,7 @@
         <v>1</v>
       </c>
       <c r="G6" t="n">
-        <v>393.6594</v>
+        <v>475.0077</v>
       </c>
     </row>
     <row r="7">
@@ -597,9 +597,7 @@
       <c r="F7" t="b">
         <v>0</v>
       </c>
-      <c r="G7" t="n">
-        <v>1528.1643</v>
-      </c>
+      <c r="G7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -621,7 +619,7 @@
         <v>0</v>
       </c>
       <c r="G8" t="n">
-        <v>506.3655</v>
+        <v>1528.1643</v>
       </c>
     </row>
     <row r="9">
@@ -644,7 +642,7 @@
         <v>1</v>
       </c>
       <c r="G9" t="n">
-        <v>357.6029</v>
+        <v>498.9721</v>
       </c>
     </row>
     <row r="10">
@@ -667,7 +665,7 @@
         <v>1</v>
       </c>
       <c r="G10" t="n">
-        <v>427.0394</v>
+        <v>543.1409</v>
       </c>
     </row>
     <row r="11">
@@ -690,7 +688,7 @@
         <v>1</v>
       </c>
       <c r="G11" t="n">
-        <v>485.2141</v>
+        <v>587.5444</v>
       </c>
     </row>
     <row r="12">
@@ -712,9 +710,7 @@
       <c r="F12" t="b">
         <v>0</v>
       </c>
-      <c r="G12" t="n">
-        <v>1484.4588</v>
-      </c>
+      <c r="G12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -736,7 +732,7 @@
         <v>0</v>
       </c>
       <c r="G13" t="n">
-        <v>763.6181</v>
+        <v>1484.4588</v>
       </c>
     </row>
     <row r="14">
@@ -759,7 +755,7 @@
         <v>0</v>
       </c>
       <c r="G14" t="n">
-        <v>549.7527</v>
+        <v>758.0975</v>
       </c>
     </row>
     <row r="15">
@@ -782,7 +778,7 @@
         <v>0</v>
       </c>
       <c r="G15" t="n">
-        <v>564.0014</v>
+        <v>709.4259</v>
       </c>
     </row>
     <row r="16">
@@ -805,7 +801,7 @@
         <v>1</v>
       </c>
       <c r="G16" t="n">
-        <v>589.9656</v>
+        <v>707.4215</v>
       </c>
     </row>
     <row r="17">
@@ -828,7 +824,7 @@
         <v>0</v>
       </c>
       <c r="G17" t="n">
-        <v>1470.1692</v>
+        <v>3476.0965</v>
       </c>
     </row>
     <row r="18">
@@ -851,7 +847,7 @@
         <v>0</v>
       </c>
       <c r="G18" t="n">
-        <v>979.0553</v>
+        <v>1470.1692</v>
       </c>
     </row>
     <row r="19">
@@ -874,7 +870,7 @@
         <v>0</v>
       </c>
       <c r="G19" t="n">
-        <v>754.4023999999999</v>
+        <v>975.1769</v>
       </c>
     </row>
     <row r="20">
@@ -897,7 +893,7 @@
         <v>0</v>
       </c>
       <c r="G20" t="n">
-        <v>726.0234</v>
+        <v>883.3682</v>
       </c>
     </row>
     <row r="21">
@@ -920,7 +916,7 @@
         <v>1</v>
       </c>
       <c r="G21" t="n">
-        <v>722.0327</v>
+        <v>847.4947</v>
       </c>
     </row>
     <row r="22">
@@ -943,7 +939,7 @@
         <v>0</v>
       </c>
       <c r="G22" t="n">
-        <v>1462.1736</v>
+        <v>2339.9803</v>
       </c>
     </row>
     <row r="23">
@@ -966,7 +962,7 @@
         <v>0</v>
       </c>
       <c r="G23" t="n">
-        <v>1089.9253</v>
+        <v>1462.1736</v>
       </c>
     </row>
     <row r="24">
@@ -989,7 +985,7 @@
         <v>0</v>
       </c>
       <c r="G24" t="n">
-        <v>881.8561999999999</v>
+        <v>1086.9377</v>
       </c>
     </row>
     <row r="25">
@@ -1012,7 +1008,7 @@
         <v>0</v>
       </c>
       <c r="G25" t="n">
-        <v>836.7375</v>
+        <v>989.7325</v>
       </c>
     </row>
     <row r="26">
@@ -1035,7 +1031,7 @@
         <v>1</v>
       </c>
       <c r="G26" t="n">
-        <v>817.8625</v>
+        <v>941.8753</v>
       </c>
     </row>
     <row r="27">
@@ -1058,7 +1054,7 @@
         <v>0</v>
       </c>
       <c r="G27" t="n">
-        <v>1451.3225</v>
+        <v>2009.4076</v>
       </c>
     </row>
     <row r="28">
@@ -1081,7 +1077,7 @@
         <v>0</v>
       </c>
       <c r="G28" t="n">
-        <v>1153.0033</v>
+        <v>1451.3225</v>
       </c>
     </row>
     <row r="29">
@@ -1104,7 +1100,7 @@
         <v>0</v>
       </c>
       <c r="G29" t="n">
-        <v>965.3873</v>
+        <v>1150.575</v>
       </c>
     </row>
     <row r="30">
@@ -1127,7 +1123,7 @@
         <v>0</v>
       </c>
       <c r="G30" t="n">
-        <v>914.2934</v>
+        <v>1057.9267</v>
       </c>
     </row>
     <row r="31">
@@ -1150,7 +1146,7 @@
         <v>1</v>
       </c>
       <c r="G31" t="n">
-        <v>888.0896</v>
+        <v>1006.8176</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Rebase Pareto front to Korea grid mix (Allocation LCA)
Switch LCA_METHOD to Allocation_KRmix. KR base is dirtier (100.83 vs
87.57 g/MJ), so CCS25/CCS50 no longer clear the 75.9 CORSIA line; the
compliance floor moves to 10% green NH3 + CCS50 (75.18 g/MJ). Make the
abatement anchor dynamic (cheapest compliant run via the conventional-jet
threshold) instead of hardcoded grey+CCS25, and update the on-plot label
and base self-check. Front grows 12 -> 15 points (CCS75 tail); MJSP
unchanged (LCA touches only the GHG axis). Rebase _Pareto_Front.md body
and regenerate figures/results.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Y2TBxkYTweca7jJJRCozLX
</commit_message>
<xml_diff>
--- a/Result/pareto_front.xlsx
+++ b/Result/pareto_front.xlsx
@@ -479,7 +479,7 @@
         <v>0.7925</v>
       </c>
       <c r="E2" t="n">
-        <v>87.57089999999999</v>
+        <v>100.834</v>
       </c>
       <c r="F2" t="b">
         <v>1</v>
@@ -500,14 +500,12 @@
         <v>0.8546</v>
       </c>
       <c r="E3" t="n">
-        <v>76.0094</v>
+        <v>89.9263</v>
       </c>
       <c r="F3" t="b">
         <v>1</v>
       </c>
-      <c r="G3" t="n">
-        <v>0</v>
-      </c>
+      <c r="G3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -523,14 +521,12 @@
         <v>0.9132</v>
       </c>
       <c r="E4" t="n">
-        <v>64.4372</v>
+        <v>78.98699999999999</v>
       </c>
       <c r="F4" t="b">
         <v>1</v>
       </c>
-      <c r="G4" t="n">
-        <v>159.9786</v>
-      </c>
+      <c r="G4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -546,13 +542,13 @@
         <v>1.1111</v>
       </c>
       <c r="E5" t="n">
-        <v>54.1746</v>
+        <v>69.3574</v>
       </c>
       <c r="F5" t="b">
         <v>1</v>
       </c>
       <c r="G5" t="n">
-        <v>371.1885</v>
+        <v>73.66759999999999</v>
       </c>
     </row>
     <row r="6">
@@ -569,13 +565,13 @@
         <v>1.3337</v>
       </c>
       <c r="E6" t="n">
-        <v>44.1505</v>
+        <v>59.9611</v>
       </c>
       <c r="F6" t="b">
         <v>1</v>
       </c>
       <c r="G6" t="n">
-        <v>475.0077</v>
+        <v>490.083</v>
       </c>
     </row>
     <row r="7">
@@ -592,7 +588,7 @@
         <v>0.9769</v>
       </c>
       <c r="E7" t="n">
-        <v>83.7593</v>
+        <v>97.0241</v>
       </c>
       <c r="F7" t="b">
         <v>0</v>
@@ -613,14 +609,12 @@
         <v>1.039</v>
       </c>
       <c r="E8" t="n">
-        <v>72.1978</v>
+        <v>86.1164</v>
       </c>
       <c r="F8" t="b">
         <v>0</v>
       </c>
-      <c r="G8" t="n">
-        <v>1528.1643</v>
-      </c>
+      <c r="G8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -636,13 +630,13 @@
         <v>1.0976</v>
       </c>
       <c r="E9" t="n">
-        <v>60.6256</v>
+        <v>75.1771</v>
       </c>
       <c r="F9" t="b">
         <v>1</v>
       </c>
       <c r="G9" t="n">
-        <v>498.9721</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10">
@@ -659,13 +653,13 @@
         <v>1.2956</v>
       </c>
       <c r="E10" t="n">
-        <v>50.363</v>
+        <v>65.5475</v>
       </c>
       <c r="F10" t="b">
         <v>1</v>
       </c>
       <c r="G10" t="n">
-        <v>543.1409</v>
+        <v>649.4063</v>
       </c>
     </row>
     <row r="11">
@@ -682,13 +676,13 @@
         <v>1.5181</v>
       </c>
       <c r="E11" t="n">
-        <v>40.3389</v>
+        <v>56.1512</v>
       </c>
       <c r="F11" t="b">
         <v>1</v>
       </c>
       <c r="G11" t="n">
-        <v>587.5444</v>
+        <v>698.0967000000001</v>
       </c>
     </row>
     <row r="12">
@@ -705,7 +699,7 @@
         <v>1.2404</v>
       </c>
       <c r="E12" t="n">
-        <v>78.04179999999999</v>
+        <v>91.30929999999999</v>
       </c>
       <c r="F12" t="b">
         <v>0</v>
@@ -726,14 +720,12 @@
         <v>1.3024</v>
       </c>
       <c r="E13" t="n">
-        <v>66.4803</v>
+        <v>80.4016</v>
       </c>
       <c r="F13" t="b">
         <v>0</v>
       </c>
-      <c r="G13" t="n">
-        <v>1484.4588</v>
-      </c>
+      <c r="G13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -749,13 +741,13 @@
         <v>1.361</v>
       </c>
       <c r="E14" t="n">
-        <v>54.9081</v>
+        <v>69.4623</v>
       </c>
       <c r="F14" t="b">
         <v>0</v>
       </c>
       <c r="G14" t="n">
-        <v>758.0975</v>
+        <v>1455.9979</v>
       </c>
     </row>
     <row r="15">
@@ -772,13 +764,13 @@
         <v>1.559</v>
       </c>
       <c r="E15" t="n">
-        <v>44.6455</v>
+        <v>59.8327</v>
       </c>
       <c r="F15" t="b">
         <v>0</v>
       </c>
       <c r="G15" t="n">
-        <v>709.4259</v>
+        <v>949.8094</v>
       </c>
     </row>
     <row r="16">
@@ -795,13 +787,13 @@
         <v>1.7815</v>
       </c>
       <c r="E16" t="n">
-        <v>34.6214</v>
+        <v>50.4364</v>
       </c>
       <c r="F16" t="b">
         <v>1</v>
       </c>
       <c r="G16" t="n">
-        <v>707.4215</v>
+        <v>873.1624</v>
       </c>
     </row>
     <row r="17">
@@ -818,14 +810,12 @@
         <v>1.6796</v>
       </c>
       <c r="E17" t="n">
-        <v>68.5127</v>
+        <v>81.7847</v>
       </c>
       <c r="F17" t="b">
         <v>0</v>
       </c>
-      <c r="G17" t="n">
-        <v>3476.0965</v>
-      </c>
+      <c r="G17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -841,13 +831,13 @@
         <v>1.7416</v>
       </c>
       <c r="E18" t="n">
-        <v>56.9512</v>
+        <v>70.877</v>
       </c>
       <c r="F18" t="b">
         <v>0</v>
       </c>
       <c r="G18" t="n">
-        <v>1470.1692</v>
+        <v>4730.6839</v>
       </c>
     </row>
     <row r="19">
@@ -864,13 +854,13 @@
         <v>1.8002</v>
       </c>
       <c r="E19" t="n">
-        <v>45.379</v>
+        <v>59.9377</v>
       </c>
       <c r="F19" t="b">
         <v>0</v>
       </c>
       <c r="G19" t="n">
-        <v>975.1769</v>
+        <v>1456.3467</v>
       </c>
     </row>
     <row r="20">
@@ -887,13 +877,13 @@
         <v>1.9982</v>
       </c>
       <c r="E20" t="n">
-        <v>35.1164</v>
+        <v>50.3081</v>
       </c>
       <c r="F20" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G20" t="n">
-        <v>883.3682</v>
+        <v>1143.8894</v>
       </c>
     </row>
     <row r="21">
@@ -910,13 +900,13 @@
         <v>2.2207</v>
       </c>
       <c r="E21" t="n">
-        <v>25.0923</v>
+        <v>40.9118</v>
       </c>
       <c r="F21" t="b">
         <v>1</v>
       </c>
       <c r="G21" t="n">
-        <v>847.4947</v>
+        <v>1035.3268</v>
       </c>
     </row>
     <row r="22">
@@ -933,13 +923,13 @@
         <v>2.1159</v>
       </c>
       <c r="E22" t="n">
-        <v>58.9837</v>
+        <v>72.26000000000001</v>
       </c>
       <c r="F22" t="b">
         <v>0</v>
       </c>
       <c r="G22" t="n">
-        <v>2339.9803</v>
+        <v>11025.9745</v>
       </c>
     </row>
     <row r="23">
@@ -956,13 +946,13 @@
         <v>2.1779</v>
       </c>
       <c r="E23" t="n">
-        <v>47.4222</v>
+        <v>61.3523</v>
       </c>
       <c r="F23" t="b">
         <v>0</v>
       </c>
       <c r="G23" t="n">
-        <v>1462.1736</v>
+        <v>2468.2752</v>
       </c>
     </row>
     <row r="24">
@@ -979,13 +969,13 @@
         <v>2.2365</v>
       </c>
       <c r="E24" t="n">
-        <v>35.85</v>
+        <v>50.413</v>
       </c>
       <c r="F24" t="b">
         <v>0</v>
       </c>
       <c r="G24" t="n">
-        <v>1086.9377</v>
+        <v>1452.6958</v>
       </c>
     </row>
     <row r="25">
@@ -1002,13 +992,13 @@
         <v>2.4345</v>
       </c>
       <c r="E25" t="n">
-        <v>25.5874</v>
+        <v>40.7834</v>
       </c>
       <c r="F25" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G25" t="n">
-        <v>989.7325</v>
+        <v>1227.7896</v>
       </c>
     </row>
     <row r="26">
@@ -1025,13 +1015,13 @@
         <v>2.657</v>
       </c>
       <c r="E26" t="n">
-        <v>15.5633</v>
+        <v>31.3871</v>
       </c>
       <c r="F26" t="b">
         <v>1</v>
       </c>
       <c r="G26" t="n">
-        <v>941.8753</v>
+        <v>1124.8372</v>
       </c>
     </row>
     <row r="27">
@@ -1048,13 +1038,13 @@
         <v>2.5439</v>
       </c>
       <c r="E27" t="n">
-        <v>49.4546</v>
+        <v>62.7354</v>
       </c>
       <c r="F27" t="b">
         <v>0</v>
       </c>
       <c r="G27" t="n">
-        <v>2009.4076</v>
+        <v>3671.7786</v>
       </c>
     </row>
     <row r="28">
@@ -1071,13 +1061,13 @@
         <v>2.606</v>
       </c>
       <c r="E28" t="n">
-        <v>37.8931</v>
+        <v>51.8277</v>
       </c>
       <c r="F28" t="b">
         <v>0</v>
       </c>
       <c r="G28" t="n">
-        <v>1451.3225</v>
+        <v>2040.4319</v>
       </c>
     </row>
     <row r="29">
@@ -1094,13 +1084,13 @@
         <v>2.6646</v>
       </c>
       <c r="E29" t="n">
-        <v>26.3209</v>
+        <v>40.8884</v>
       </c>
       <c r="F29" t="b">
         <v>0</v>
       </c>
       <c r="G29" t="n">
-        <v>1150.575</v>
+        <v>1443.4548</v>
       </c>
     </row>
     <row r="30">
@@ -1117,13 +1107,13 @@
         <v>2.8625</v>
       </c>
       <c r="E30" t="n">
-        <v>16.0583</v>
+        <v>31.2588</v>
       </c>
       <c r="F30" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G30" t="n">
-        <v>1057.9267</v>
+        <v>1269.3505</v>
       </c>
     </row>
     <row r="31">
@@ -1140,13 +1130,13 @@
         <v>3.0851</v>
       </c>
       <c r="E31" t="n">
-        <v>6.0342</v>
+        <v>21.8625</v>
       </c>
       <c r="F31" t="b">
         <v>1</v>
       </c>
       <c r="G31" t="n">
-        <v>1006.8176</v>
+        <v>1177.4658</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Rebase Pareto abatement anchor onto CCS 60% base
Replace the dynamic cheapest-compliant floor (NH3 10% + CCS 50%) with a
fixed CCS 60% base in tea_pareto_front.py main(): anchor_ghg by linear
interp of CCS050/CCS075 at c=0.60 (75.14 g/MJ), anchor_mjsp from
economic_analysis at ccs_portion=0.60 (0.977 $/L). Cells at/above the base
GHG -> NaN. Add CORSIA self-check + anchor print.

Base premium drops 1.098 -> 0.977 $/L, so all abatement costs rise:
cheapest step below base = grey+CCS75 at 733 $/t (was 74). Ranking
unchanged: CCS first, ammonia last.

Update _Pareto_Front.md section 5 (heading/prose/table/contour caption),
correct the section 7 forward-note, add log entry 2026-09-30 (update 3).
Regenerate pareto_front.png, pareto_abatement_contour_compliance.png,
pareto_front.xlsx, pareto_front_sensitivity.xlsx.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Result/pareto_front.xlsx
+++ b/Result/pareto_front.xlsx
@@ -548,7 +548,7 @@
         <v>1</v>
       </c>
       <c r="G5" t="n">
-        <v>73.66759999999999</v>
+        <v>732.8276</v>
       </c>
     </row>
     <row r="6">
@@ -571,7 +571,7 @@
         <v>1</v>
       </c>
       <c r="G6" t="n">
-        <v>490.083</v>
+        <v>742.2204</v>
       </c>
     </row>
     <row r="7">
@@ -635,9 +635,7 @@
       <c r="F9" t="b">
         <v>1</v>
       </c>
-      <c r="G9" t="n">
-        <v>0</v>
-      </c>
+      <c r="G9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -659,7 +657,7 @@
         <v>1</v>
       </c>
       <c r="G10" t="n">
-        <v>649.4063</v>
+        <v>1049.1549</v>
       </c>
     </row>
     <row r="11">
@@ -682,7 +680,7 @@
         <v>1</v>
       </c>
       <c r="G11" t="n">
-        <v>698.0967000000001</v>
+        <v>900.093</v>
       </c>
     </row>
     <row r="12">
@@ -747,7 +745,7 @@
         <v>0</v>
       </c>
       <c r="G14" t="n">
-        <v>1455.9979</v>
+        <v>2137.5822</v>
       </c>
     </row>
     <row r="15">
@@ -770,7 +768,7 @@
         <v>0</v>
       </c>
       <c r="G15" t="n">
-        <v>949.8094</v>
+        <v>1201.0932</v>
       </c>
     </row>
     <row r="16">
@@ -793,7 +791,7 @@
         <v>1</v>
       </c>
       <c r="G16" t="n">
-        <v>873.1624</v>
+        <v>1028.7184</v>
       </c>
     </row>
     <row r="17">
@@ -837,7 +835,7 @@
         <v>0</v>
       </c>
       <c r="G18" t="n">
-        <v>4730.6839</v>
+        <v>5670.989</v>
       </c>
     </row>
     <row r="19">
@@ -860,7 +858,7 @@
         <v>0</v>
       </c>
       <c r="G19" t="n">
-        <v>1456.3467</v>
+        <v>1710.765</v>
       </c>
     </row>
     <row r="20">
@@ -883,7 +881,7 @@
         <v>1</v>
       </c>
       <c r="G20" t="n">
-        <v>1143.8894</v>
+        <v>1299.0989</v>
       </c>
     </row>
     <row r="21">
@@ -906,7 +904,7 @@
         <v>1</v>
       </c>
       <c r="G21" t="n">
-        <v>1035.3268</v>
+        <v>1147.7892</v>
       </c>
     </row>
     <row r="22">
@@ -929,7 +927,7 @@
         <v>0</v>
       </c>
       <c r="G22" t="n">
-        <v>11025.9745</v>
+        <v>12510.5249</v>
       </c>
     </row>
     <row r="23">
@@ -952,7 +950,7 @@
         <v>0</v>
       </c>
       <c r="G23" t="n">
-        <v>2468.2752</v>
+        <v>2751.8888</v>
       </c>
     </row>
     <row r="24">
@@ -975,7 +973,7 @@
         <v>0</v>
       </c>
       <c r="G24" t="n">
-        <v>1452.6958</v>
+        <v>1609.0886</v>
       </c>
     </row>
     <row r="25">
@@ -998,7 +996,7 @@
         <v>1</v>
       </c>
       <c r="G25" t="n">
-        <v>1227.7896</v>
+        <v>1340.0669</v>
       </c>
     </row>
     <row r="26">
@@ -1021,7 +1019,7 @@
         <v>1</v>
       </c>
       <c r="G26" t="n">
-        <v>1124.8372</v>
+        <v>1212.9005</v>
       </c>
     </row>
     <row r="27">
@@ -1044,7 +1042,7 @@
         <v>0</v>
       </c>
       <c r="G27" t="n">
-        <v>3671.7786</v>
+        <v>3991.1007</v>
       </c>
     </row>
     <row r="28">
@@ -1067,7 +1065,7 @@
         <v>0</v>
       </c>
       <c r="G28" t="n">
-        <v>2040.4319</v>
+        <v>2207.3755</v>
       </c>
     </row>
     <row r="29">
@@ -1090,7 +1088,7 @@
         <v>0</v>
       </c>
       <c r="G29" t="n">
-        <v>1443.4548</v>
+        <v>1556.3405</v>
       </c>
     </row>
     <row r="30">
@@ -1113,7 +1111,7 @@
         <v>1</v>
       </c>
       <c r="G30" t="n">
-        <v>1269.3505</v>
+        <v>1357.2945</v>
       </c>
     </row>
     <row r="31">
@@ -1136,7 +1134,7 @@
         <v>1</v>
       </c>
       <c r="G31" t="n">
-        <v>1177.4658</v>
+        <v>1249.8257</v>
       </c>
     </row>
   </sheetData>

</xml_diff>